<commit_message>
vFinal twin: avisuite palette, names cleared
</commit_message>
<xml_diff>
--- a/uploads/inbox/SPV_ROSTER_TEMPLATE_AVISUITE_COLORS.xlsx
+++ b/uploads/inbox/SPV_ROSTER_TEMPLATE_AVISUITE_COLORS.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROSTER" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROSTER'!$A$1:$AI$88</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROSTER'!$A$1:$AI$89</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="36">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -118,7 +118,75 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
       <color rgb="00196B24"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="001A56DB"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="005521B5"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="000E7490"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -126,10 +194,6 @@
       <b val="1"/>
       <color rgb="00F9FAFB"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Times New Roman"/>
@@ -174,7 +238,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="28">
     <fill>
       <patternFill/>
     </fill>
@@ -243,6 +307,41 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0CECE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEBFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFFAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -747,7 +846,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1063,10 +1162,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1093,32 +1198,59 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="23" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="24" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="26" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="27" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1130,76 +1262,46 @@
   <cellStyles count="1">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="27">
     <dxf>
-      <font>
-        <name val="Times New Roman"/>
-        <b val="1"/>
-        <color rgb="0092400E"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="00FEF3C7"/>
+          <bgColor rgb="FFFFFF99"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <name val="Times New Roman"/>
-        <b val="1"/>
-        <color rgb="001A56DB"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="00DBEAFE"/>
+          <bgColor theme="4" tint="0.7999816888943144"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <name val="Times New Roman"/>
-        <b val="1"/>
-        <color rgb="00065F46"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="00D1FAE5"/>
+          <bgColor theme="3" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <name val="Times New Roman"/>
-        <b val="1"/>
-        <color rgb="006B7280"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="00F3F4F6"/>
+          <bgColor theme="0" tint="-0.249946592608417"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <name val="Times New Roman"/>
-        <b val="1"/>
-        <color rgb="000E7490"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="00CFFAFE"/>
+          <bgColor theme="9" tint="0.3999450666829432"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <name val="Times New Roman"/>
-        <b val="1"/>
-        <color rgb="005521B5"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="00EDEBFE"/>
+          <bgColor theme="8" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1242,6 +1344,66 @@
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.5999633777886288"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Times New Roman"/>
+        <b val="1"/>
+        <color rgb="0092400E"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00FEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Times New Roman"/>
+        <b val="1"/>
+        <color rgb="001A56DB"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00DBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Times New Roman"/>
+        <b val="1"/>
+        <color rgb="00065F46"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00D1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Times New Roman"/>
+        <b val="1"/>
+        <color rgb="005521B5"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00EDEBFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Times New Roman"/>
+        <b val="1"/>
+        <color rgb="000E7490"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00CFFAFE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1338,6 +1500,20 @@
       <fill>
         <patternFill>
           <bgColor rgb="00FEF9C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00DBEDD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00A1BFCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1735,7 +1911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AP87"/>
+  <dimension ref="A1:AP88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1856,282 +2032,282 @@
           <t>CREW 1</t>
         </is>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="109">
         <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,1),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="109">
         <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,2),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="109">
         <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,3),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="109">
         <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,4),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="109">
         <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,5),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="109">
         <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,6),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="109">
         <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,7),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="L3" s="1">
+      <c r="L3" s="109">
         <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,8),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="M3" s="1">
+      <c r="M3" s="109">
         <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,9),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="109">
         <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,10),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="109">
         <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,11),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="109">
         <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,12),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="109">
         <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,13),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="109">
         <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,14),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="109">
         <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,15),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="T3" s="1">
+      <c r="T3" s="109">
         <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,16),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="U3" s="1">
+      <c r="U3" s="109">
         <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,17),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="V3" s="1">
+      <c r="V3" s="109">
         <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,18),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="W3" s="1">
+      <c r="W3" s="109">
         <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,19),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="X3" s="1">
+      <c r="X3" s="109">
         <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,20),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Y3" s="1">
+      <c r="Y3" s="109">
         <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,21),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Z3" s="1">
+      <c r="Z3" s="109">
         <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,22),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AA3" s="1">
+      <c r="AA3" s="109">
         <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,23),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AB3" s="1">
+      <c r="AB3" s="109">
         <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,24),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AC3" s="1">
+      <c r="AC3" s="109">
         <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,25),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AD3" s="1">
+      <c r="AD3" s="109">
         <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,26),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AE3" s="1">
+      <c r="AE3" s="109">
         <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,27),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AF3" s="1">
+      <c r="AF3" s="109">
         <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,28),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AG3" s="1">
+      <c r="AG3" s="109">
         <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,29),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AH3" s="24">
+      <c r="AH3" s="109">
         <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,30),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AI3" s="21">
+      <c r="AI3" s="109">
         <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,31),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AK3" s="109" t="inlineStr">
+      <c r="AK3" s="110" t="inlineStr">
         <is>
           <t>ROSTER PERIOD</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A4" s="110" t="n"/>
-      <c r="E4" s="2">
+      <c r="A4" s="111" t="n"/>
+      <c r="E4" s="112">
         <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),1,"")</f>
         <v/>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="112">
         <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),2,"")</f>
         <v/>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="112">
         <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),3,"")</f>
         <v/>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="112">
         <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),4,"")</f>
         <v/>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="112">
         <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),5,"")</f>
         <v/>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="112">
         <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),6,"")</f>
         <v/>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="112">
         <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),7,"")</f>
         <v/>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="112">
         <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),8,"")</f>
         <v/>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="112">
         <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),9,"")</f>
         <v/>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="112">
         <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),10,"")</f>
         <v/>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="112">
         <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),11,"")</f>
         <v/>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="112">
         <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),12,"")</f>
         <v/>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="112">
         <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),13,"")</f>
         <v/>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="112">
         <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),14,"")</f>
         <v/>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="112">
         <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),15,"")</f>
         <v/>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="112">
         <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),16,"")</f>
         <v/>
       </c>
-      <c r="U4" s="2">
+      <c r="U4" s="112">
         <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),17,"")</f>
         <v/>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="112">
         <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),18,"")</f>
         <v/>
       </c>
-      <c r="W4" s="2">
+      <c r="W4" s="112">
         <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),19,"")</f>
         <v/>
       </c>
-      <c r="X4" s="2">
+      <c r="X4" s="112">
         <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),20,"")</f>
         <v/>
       </c>
-      <c r="Y4" s="2">
+      <c r="Y4" s="112">
         <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),21,"")</f>
         <v/>
       </c>
-      <c r="Z4" s="2">
+      <c r="Z4" s="112">
         <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),22,"")</f>
         <v/>
       </c>
-      <c r="AA4" s="2">
+      <c r="AA4" s="112">
         <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),23,"")</f>
         <v/>
       </c>
-      <c r="AB4" s="2">
+      <c r="AB4" s="112">
         <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),24,"")</f>
         <v/>
       </c>
-      <c r="AC4" s="2">
+      <c r="AC4" s="112">
         <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),25,"")</f>
         <v/>
       </c>
-      <c r="AD4" s="2">
+      <c r="AD4" s="112">
         <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),26,"")</f>
         <v/>
       </c>
-      <c r="AE4" s="2">
+      <c r="AE4" s="112">
         <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),27,"")</f>
         <v/>
       </c>
-      <c r="AF4" s="2">
+      <c r="AF4" s="112">
         <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),28,"")</f>
         <v/>
       </c>
-      <c r="AG4" s="2">
+      <c r="AG4" s="112">
         <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),29,"")</f>
         <v/>
       </c>
-      <c r="AH4" s="25">
+      <c r="AH4" s="112">
         <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),30,"")</f>
         <v/>
       </c>
-      <c r="AI4" s="22">
+      <c r="AI4" s="112">
         <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),31,"")</f>
         <v/>
       </c>
-      <c r="AK4" s="111" t="inlineStr">
+      <c r="AK4" s="113" t="inlineStr">
         <is>
           <t>MONTH</t>
         </is>
       </c>
-      <c r="AL4" s="112" t="inlineStr">
+      <c r="AL4" s="114" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="AM4" s="135" t="n"/>
-      <c r="AN4" s="136" t="n"/>
+      <c r="AM4" s="146" t="n"/>
+      <c r="AN4" s="147" t="n"/>
     </row>
     <row r="5" ht="16.2" customHeight="1" thickBot="1">
       <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="33" t="n"/>
-      <c r="C5" s="33" t="n"/>
-      <c r="D5" s="34" t="n"/>
+      <c r="B5" s="37" t="n"/>
+      <c r="C5" s="37" t="n"/>
+      <c r="D5" s="40" t="n"/>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="7" t="n"/>
@@ -2163,24 +2339,24 @@
       <c r="AG5" s="6" t="n"/>
       <c r="AH5" s="26" t="n"/>
       <c r="AI5" s="23" t="n"/>
-      <c r="AK5" s="111" t="inlineStr">
+      <c r="AK5" s="113" t="inlineStr">
         <is>
           <t>YEAR</t>
         </is>
       </c>
-      <c r="AL5" s="112" t="n">
+      <c r="AL5" s="114" t="n">
         <v>2026</v>
       </c>
-      <c r="AM5" s="135" t="n"/>
-      <c r="AN5" s="136" t="n"/>
+      <c r="AM5" s="146" t="n"/>
+      <c r="AN5" s="147" t="n"/>
     </row>
     <row r="6" ht="16.2" customHeight="1" thickBot="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="33" t="n"/>
-      <c r="C6" s="33" t="n"/>
-      <c r="D6" s="33" t="n"/>
+      <c r="B6" s="37" t="n"/>
+      <c r="C6" s="37" t="n"/>
+      <c r="D6" s="37" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="7" t="n"/>
@@ -2212,7 +2388,7 @@
       <c r="AG6" s="6" t="n"/>
       <c r="AH6" s="26" t="n"/>
       <c r="AI6" s="23" t="n"/>
-      <c r="AK6" s="113" t="inlineStr">
+      <c r="AK6" s="115" t="inlineStr">
         <is>
           <t>type JUL / JULY / 7</t>
         </is>
@@ -2222,9 +2398,9 @@
       <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="35" t="n"/>
-      <c r="C7" s="33" t="n"/>
-      <c r="D7" s="33" t="n"/>
+      <c r="B7" s="36" t="n"/>
+      <c r="C7" s="37" t="n"/>
+      <c r="D7" s="37" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="7" t="n"/>
@@ -2261,9 +2437,9 @@
       <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="33" t="n"/>
-      <c r="C8" s="33" t="n"/>
-      <c r="D8" s="33" t="n"/>
+      <c r="B8" s="37" t="n"/>
+      <c r="C8" s="37" t="n"/>
+      <c r="D8" s="37" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="7" t="n"/>
@@ -2339,9 +2515,9 @@
       <c r="A10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="38" t="n"/>
-      <c r="C10" s="38" t="n"/>
-      <c r="D10" s="38" t="n"/>
+      <c r="B10" s="37" t="n"/>
+      <c r="C10" s="37" t="n"/>
+      <c r="D10" s="37" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="7" t="n"/>
@@ -2378,9 +2554,9 @@
       <c r="A11" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="38" t="n"/>
-      <c r="C11" s="38" t="n"/>
-      <c r="D11" s="38" t="n"/>
+      <c r="B11" s="37" t="n"/>
+      <c r="C11" s="37" t="n"/>
+      <c r="D11" s="37" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="7" t="n"/>
@@ -2417,9 +2593,9 @@
       <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="38" t="n"/>
-      <c r="C12" s="38" t="n"/>
-      <c r="D12" s="38" t="n"/>
+      <c r="B12" s="37" t="n"/>
+      <c r="C12" s="37" t="n"/>
+      <c r="D12" s="37" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="7" t="n"/>
@@ -2456,9 +2632,9 @@
       <c r="A13" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="38" t="n"/>
-      <c r="C13" s="38" t="n"/>
-      <c r="D13" s="38" t="n"/>
+      <c r="B13" s="37" t="n"/>
+      <c r="C13" s="37" t="n"/>
+      <c r="D13" s="37" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="7" t="n"/>
@@ -2495,9 +2671,9 @@
       <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="38" t="n"/>
-      <c r="C14" s="38" t="n"/>
-      <c r="D14" s="38" t="n"/>
+      <c r="B14" s="37" t="n"/>
+      <c r="C14" s="37" t="n"/>
+      <c r="D14" s="37" t="n"/>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
       <c r="G14" s="11" t="n"/>
@@ -2534,9 +2710,9 @@
       <c r="A15" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="38" t="n"/>
-      <c r="C15" s="38" t="n"/>
-      <c r="D15" s="38" t="n"/>
+      <c r="B15" s="37" t="n"/>
+      <c r="C15" s="37" t="n"/>
+      <c r="D15" s="37" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="7" t="n"/>
@@ -2786,85 +2962,271 @@
           <t>CREW 2</t>
         </is>
       </c>
-      <c r="B22" s="114" t="n"/>
-      <c r="C22" s="114" t="n"/>
-      <c r="D22" s="114" t="n"/>
-      <c r="E22" s="30" t="n"/>
-      <c r="F22" s="30" t="n"/>
-      <c r="G22" s="30" t="n"/>
-      <c r="H22" s="30" t="n"/>
-      <c r="I22" s="30" t="n"/>
-      <c r="J22" s="30" t="n"/>
-      <c r="K22" s="30" t="n"/>
-      <c r="L22" s="30" t="n"/>
-      <c r="M22" s="30" t="n"/>
-      <c r="N22" s="30" t="n"/>
-      <c r="O22" s="30" t="n"/>
-      <c r="P22" s="30" t="n"/>
-      <c r="Q22" s="30" t="n"/>
-      <c r="R22" s="30" t="n"/>
-      <c r="S22" s="30" t="n"/>
-      <c r="T22" s="30" t="n"/>
-      <c r="U22" s="30" t="n"/>
-      <c r="V22" s="30" t="n"/>
-      <c r="W22" s="30" t="n"/>
-      <c r="X22" s="30" t="n"/>
-      <c r="Y22" s="30" t="n"/>
-      <c r="Z22" s="30" t="n"/>
-      <c r="AA22" s="30" t="n"/>
-      <c r="AB22" s="30" t="n"/>
-      <c r="AC22" s="30" t="n"/>
-      <c r="AD22" s="30" t="n"/>
-      <c r="AE22" s="30" t="n"/>
-      <c r="AF22" s="30" t="n"/>
-      <c r="AG22" s="30" t="n"/>
-      <c r="AH22" s="30" t="n"/>
-      <c r="AI22" s="31" t="n"/>
+      <c r="B22" s="116" t="n"/>
+      <c r="C22" s="116" t="n"/>
+      <c r="D22" s="116" t="n"/>
+      <c r="E22" s="109">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,1),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="109">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,2),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="109">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,3),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="109">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,4),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="109">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,5),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="109">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,6),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="109">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,7),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="109">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,8),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="109">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,9),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="109">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,10),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="109">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,11),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="109">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,12),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="109">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,13),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="109">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,14),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="S22" s="109">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,15),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="T22" s="109">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,16),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="U22" s="109">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,17),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="V22" s="109">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,18),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="W22" s="109">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,19),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="X22" s="109">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,20),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Y22" s="109">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,21),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Z22" s="109">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,22),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AA22" s="109">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,23),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AB22" s="109">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,24),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AC22" s="109">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,25),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AD22" s="109">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,26),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AE22" s="109">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,27),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AF22" s="109">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,28),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AG22" s="109">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,29),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AH22" s="109">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,30),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AI22" s="109">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,31),"ddd"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A23" s="115" t="n"/>
-      <c r="B23" s="116" t="n"/>
-      <c r="C23" s="116" t="n"/>
-      <c r="D23" s="116" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="4" t="n"/>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="n"/>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="n"/>
-      <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
-      <c r="W23" s="2" t="n"/>
-      <c r="X23" s="2" t="n"/>
-      <c r="Y23" s="2" t="n"/>
-      <c r="Z23" s="2" t="n"/>
-      <c r="AA23" s="2" t="n"/>
-      <c r="AB23" s="2" t="n"/>
-      <c r="AC23" s="2" t="n"/>
-      <c r="AD23" s="2" t="n"/>
-      <c r="AE23" s="2" t="n"/>
-      <c r="AF23" s="2" t="n"/>
-      <c r="AG23" s="2" t="n"/>
-      <c r="AH23" s="2" t="n"/>
-      <c r="AI23" s="25" t="n"/>
+      <c r="A23" s="117" t="n"/>
+      <c r="B23" s="118" t="n"/>
+      <c r="C23" s="118" t="n"/>
+      <c r="D23" s="118" t="n"/>
+      <c r="E23" s="112">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),1,"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="112">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),2,"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="112">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),3,"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="112">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),4,"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="112">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),5,"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="112">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),6,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="112">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),7,"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="112">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),8,"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="112">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),9,"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="112">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),10,"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="112">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),11,"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="112">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),12,"")</f>
+        <v/>
+      </c>
+      <c r="Q23" s="112">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),13,"")</f>
+        <v/>
+      </c>
+      <c r="R23" s="112">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),14,"")</f>
+        <v/>
+      </c>
+      <c r="S23" s="112">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),15,"")</f>
+        <v/>
+      </c>
+      <c r="T23" s="112">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),16,"")</f>
+        <v/>
+      </c>
+      <c r="U23" s="112">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),17,"")</f>
+        <v/>
+      </c>
+      <c r="V23" s="112">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),18,"")</f>
+        <v/>
+      </c>
+      <c r="W23" s="112">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),19,"")</f>
+        <v/>
+      </c>
+      <c r="X23" s="112">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),20,"")</f>
+        <v/>
+      </c>
+      <c r="Y23" s="112">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),21,"")</f>
+        <v/>
+      </c>
+      <c r="Z23" s="112">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),22,"")</f>
+        <v/>
+      </c>
+      <c r="AA23" s="112">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),23,"")</f>
+        <v/>
+      </c>
+      <c r="AB23" s="112">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),24,"")</f>
+        <v/>
+      </c>
+      <c r="AC23" s="112">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),25,"")</f>
+        <v/>
+      </c>
+      <c r="AD23" s="112">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),26,"")</f>
+        <v/>
+      </c>
+      <c r="AE23" s="112">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),27,"")</f>
+        <v/>
+      </c>
+      <c r="AF23" s="112">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),28,"")</f>
+        <v/>
+      </c>
+      <c r="AG23" s="112">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),29,"")</f>
+        <v/>
+      </c>
+      <c r="AH23" s="112">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),30,"")</f>
+        <v/>
+      </c>
+      <c r="AI23" s="112">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),31,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="16.2" customHeight="1" thickBot="1">
       <c r="A24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B24" s="33" t="n"/>
-      <c r="C24" s="33" t="n"/>
-      <c r="D24" s="33" t="n"/>
+      <c r="B24" s="37" t="n"/>
+      <c r="C24" s="37" t="n"/>
+      <c r="D24" s="37" t="n"/>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="n"/>
@@ -2901,9 +3263,9 @@
       <c r="A25" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B25" s="33" t="n"/>
-      <c r="C25" s="33" t="n"/>
-      <c r="D25" s="33" t="n"/>
+      <c r="B25" s="37" t="n"/>
+      <c r="C25" s="37" t="n"/>
+      <c r="D25" s="37" t="n"/>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
@@ -3057,9 +3419,9 @@
       <c r="A29" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B29" s="38" t="n"/>
-      <c r="C29" s="38" t="n"/>
-      <c r="D29" s="38" t="n"/>
+      <c r="B29" s="37" t="n"/>
+      <c r="C29" s="37" t="n"/>
+      <c r="D29" s="37" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
       <c r="G29" s="6" t="n"/>
@@ -3096,9 +3458,9 @@
       <c r="A30" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B30" s="38" t="n"/>
-      <c r="C30" s="38" t="n"/>
-      <c r="D30" s="38" t="n"/>
+      <c r="B30" s="37" t="n"/>
+      <c r="C30" s="37" t="n"/>
+      <c r="D30" s="37" t="n"/>
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
       <c r="G30" s="6" t="n"/>
@@ -3135,9 +3497,9 @@
       <c r="A31" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B31" s="38" t="n"/>
-      <c r="C31" s="38" t="n"/>
-      <c r="D31" s="38" t="n"/>
+      <c r="B31" s="37" t="n"/>
+      <c r="C31" s="37" t="n"/>
+      <c r="D31" s="37" t="n"/>
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
       <c r="G31" s="6" t="n"/>
@@ -3174,9 +3536,9 @@
       <c r="A32" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B32" s="38" t="n"/>
-      <c r="C32" s="38" t="n"/>
-      <c r="D32" s="38" t="n"/>
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="37" t="n"/>
+      <c r="D32" s="37" t="n"/>
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
       <c r="G32" s="6" t="n"/>
@@ -3213,9 +3575,9 @@
       <c r="A33" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B33" s="38" t="n"/>
-      <c r="C33" s="38" t="n"/>
-      <c r="D33" s="38" t="n"/>
+      <c r="B33" s="37" t="n"/>
+      <c r="C33" s="37" t="n"/>
+      <c r="D33" s="37" t="n"/>
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
       <c r="G33" s="6" t="n"/>
@@ -3252,9 +3614,9 @@
       <c r="A34" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B34" s="38" t="n"/>
-      <c r="C34" s="38" t="n"/>
-      <c r="D34" s="38" t="n"/>
+      <c r="B34" s="37" t="n"/>
+      <c r="C34" s="37" t="n"/>
+      <c r="D34" s="37" t="n"/>
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
       <c r="G34" s="6" t="n"/>
@@ -3291,9 +3653,9 @@
       <c r="A35" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B35" s="38" t="n"/>
-      <c r="C35" s="38" t="n"/>
-      <c r="D35" s="38" t="n"/>
+      <c r="B35" s="37" t="n"/>
+      <c r="C35" s="37" t="n"/>
+      <c r="D35" s="37" t="n"/>
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
       <c r="G35" s="6" t="n"/>
@@ -3330,9 +3692,9 @@
       <c r="A36" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B36" s="38" t="n"/>
-      <c r="C36" s="38" t="n"/>
-      <c r="D36" s="38" t="n"/>
+      <c r="B36" s="37" t="n"/>
+      <c r="C36" s="37" t="n"/>
+      <c r="D36" s="37" t="n"/>
       <c r="E36" s="6" t="n"/>
       <c r="F36" s="6" t="n"/>
       <c r="G36" s="6" t="n"/>
@@ -3523,82 +3885,268 @@
     </row>
     <row r="41" ht="15" customHeight="1" thickBot="1"/>
     <row r="42" ht="15" customHeight="1" thickBot="1">
-      <c r="A42" s="117" t="inlineStr">
+      <c r="A42" s="119" t="inlineStr">
         <is>
           <t>SPECIAL SHIFTING</t>
         </is>
       </c>
-      <c r="B42" s="114" t="n"/>
-      <c r="C42" s="114" t="n"/>
-      <c r="D42" s="118" t="n"/>
-      <c r="E42" s="1" t="n"/>
-      <c r="F42" s="1" t="n"/>
-      <c r="G42" s="1" t="n"/>
-      <c r="H42" s="1" t="n"/>
-      <c r="I42" s="1" t="n"/>
-      <c r="J42" s="1" t="n"/>
-      <c r="K42" s="1" t="n"/>
-      <c r="L42" s="1" t="n"/>
-      <c r="M42" s="1" t="n"/>
-      <c r="N42" s="1" t="n"/>
-      <c r="O42" s="1" t="n"/>
-      <c r="P42" s="1" t="n"/>
-      <c r="Q42" s="1" t="n"/>
-      <c r="R42" s="1" t="n"/>
-      <c r="S42" s="1" t="n"/>
-      <c r="T42" s="1" t="n"/>
-      <c r="U42" s="1" t="n"/>
-      <c r="V42" s="1" t="n"/>
-      <c r="W42" s="1" t="n"/>
-      <c r="X42" s="1" t="n"/>
-      <c r="Y42" s="1" t="n"/>
-      <c r="Z42" s="1" t="n"/>
-      <c r="AA42" s="1" t="n"/>
-      <c r="AB42" s="1" t="n"/>
-      <c r="AC42" s="1" t="n"/>
-      <c r="AD42" s="1" t="n"/>
-      <c r="AE42" s="1" t="n"/>
-      <c r="AF42" s="1" t="n"/>
-      <c r="AG42" s="1" t="n"/>
-      <c r="AH42" s="1" t="n"/>
-      <c r="AI42" s="1" t="n"/>
+      <c r="B42" s="116" t="n"/>
+      <c r="C42" s="116" t="n"/>
+      <c r="D42" s="120" t="n"/>
+      <c r="E42" s="109">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,1),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="109">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,2),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="G42" s="109">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,3),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="H42" s="109">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,4),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="I42" s="109">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,5),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="J42" s="109">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,6),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="K42" s="109">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,7),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="L42" s="109">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,8),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="M42" s="109">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,9),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="N42" s="109">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,10),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="O42" s="109">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,11),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="P42" s="109">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,12),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Q42" s="109">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,13),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="R42" s="109">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,14),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="S42" s="109">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,15),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="T42" s="109">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,16),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="U42" s="109">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,17),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="V42" s="109">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,18),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="W42" s="109">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,19),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="X42" s="109">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,20),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Y42" s="109">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,21),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Z42" s="109">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,22),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AA42" s="109">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,23),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AB42" s="109">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,24),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AC42" s="109">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,25),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AD42" s="109">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,26),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AE42" s="109">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,27),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AF42" s="109">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,28),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AG42" s="109">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,29),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AH42" s="109">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,30),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AI42" s="109">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,31),"ddd"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A43" s="115" t="n"/>
-      <c r="B43" s="116" t="n"/>
-      <c r="C43" s="116" t="n"/>
-      <c r="D43" s="119" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-      <c r="L43" s="3" t="n"/>
-      <c r="M43" s="4" t="n"/>
-      <c r="N43" s="2" t="n"/>
-      <c r="O43" s="2" t="n"/>
-      <c r="P43" s="2" t="n"/>
-      <c r="Q43" s="2" t="n"/>
-      <c r="R43" s="2" t="n"/>
-      <c r="S43" s="2" t="n"/>
-      <c r="T43" s="2" t="n"/>
-      <c r="U43" s="2" t="n"/>
-      <c r="V43" s="2" t="n"/>
-      <c r="W43" s="2" t="n"/>
-      <c r="X43" s="2" t="n"/>
-      <c r="Y43" s="2" t="n"/>
-      <c r="Z43" s="2" t="n"/>
-      <c r="AA43" s="2" t="n"/>
-      <c r="AB43" s="2" t="n"/>
-      <c r="AC43" s="2" t="n"/>
-      <c r="AD43" s="2" t="n"/>
-      <c r="AE43" s="2" t="n"/>
-      <c r="AF43" s="2" t="n"/>
-      <c r="AG43" s="2" t="n"/>
-      <c r="AH43" s="2" t="n"/>
-      <c r="AI43" s="2" t="n"/>
+      <c r="A43" s="117" t="n"/>
+      <c r="B43" s="118" t="n"/>
+      <c r="C43" s="118" t="n"/>
+      <c r="D43" s="121" t="n"/>
+      <c r="E43" s="112">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),1,"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="112">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),2,"")</f>
+        <v/>
+      </c>
+      <c r="G43" s="112">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),3,"")</f>
+        <v/>
+      </c>
+      <c r="H43" s="112">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),4,"")</f>
+        <v/>
+      </c>
+      <c r="I43" s="112">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),5,"")</f>
+        <v/>
+      </c>
+      <c r="J43" s="112">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),6,"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="112">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),7,"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="112">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),8,"")</f>
+        <v/>
+      </c>
+      <c r="M43" s="112">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),9,"")</f>
+        <v/>
+      </c>
+      <c r="N43" s="112">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),10,"")</f>
+        <v/>
+      </c>
+      <c r="O43" s="112">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),11,"")</f>
+        <v/>
+      </c>
+      <c r="P43" s="112">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),12,"")</f>
+        <v/>
+      </c>
+      <c r="Q43" s="112">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),13,"")</f>
+        <v/>
+      </c>
+      <c r="R43" s="112">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),14,"")</f>
+        <v/>
+      </c>
+      <c r="S43" s="112">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),15,"")</f>
+        <v/>
+      </c>
+      <c r="T43" s="112">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),16,"")</f>
+        <v/>
+      </c>
+      <c r="U43" s="112">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),17,"")</f>
+        <v/>
+      </c>
+      <c r="V43" s="112">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),18,"")</f>
+        <v/>
+      </c>
+      <c r="W43" s="112">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),19,"")</f>
+        <v/>
+      </c>
+      <c r="X43" s="112">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),20,"")</f>
+        <v/>
+      </c>
+      <c r="Y43" s="112">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),21,"")</f>
+        <v/>
+      </c>
+      <c r="Z43" s="112">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),22,"")</f>
+        <v/>
+      </c>
+      <c r="AA43" s="112">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),23,"")</f>
+        <v/>
+      </c>
+      <c r="AB43" s="112">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),24,"")</f>
+        <v/>
+      </c>
+      <c r="AC43" s="112">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),25,"")</f>
+        <v/>
+      </c>
+      <c r="AD43" s="112">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),26,"")</f>
+        <v/>
+      </c>
+      <c r="AE43" s="112">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),27,"")</f>
+        <v/>
+      </c>
+      <c r="AF43" s="112">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),28,"")</f>
+        <v/>
+      </c>
+      <c r="AG43" s="112">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),29,"")</f>
+        <v/>
+      </c>
+      <c r="AH43" s="112">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),30,"")</f>
+        <v/>
+      </c>
+      <c r="AI43" s="112">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),31,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="16.2" customHeight="1" thickBot="1">
       <c r="A44" s="5" t="n">
@@ -3657,82 +4205,268 @@
       <c r="O45" s="14" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
-      <c r="A46" s="117" t="inlineStr">
+      <c r="A46" s="119" t="inlineStr">
         <is>
           <t>TRANSFERRED-IN MANPOWER</t>
         </is>
       </c>
-      <c r="B46" s="114" t="n"/>
-      <c r="C46" s="114" t="n"/>
-      <c r="D46" s="118" t="n"/>
-      <c r="E46" s="1" t="n"/>
-      <c r="F46" s="1" t="n"/>
-      <c r="G46" s="1" t="n"/>
-      <c r="H46" s="1" t="n"/>
-      <c r="I46" s="1" t="n"/>
-      <c r="J46" s="1" t="n"/>
-      <c r="K46" s="1" t="n"/>
-      <c r="L46" s="1" t="n"/>
-      <c r="M46" s="1" t="n"/>
-      <c r="N46" s="1" t="n"/>
-      <c r="O46" s="1" t="n"/>
-      <c r="P46" s="1" t="n"/>
-      <c r="Q46" s="1" t="n"/>
-      <c r="R46" s="1" t="n"/>
-      <c r="S46" s="1" t="n"/>
-      <c r="T46" s="1" t="n"/>
-      <c r="U46" s="1" t="n"/>
-      <c r="V46" s="1" t="n"/>
-      <c r="W46" s="1" t="n"/>
-      <c r="X46" s="1" t="n"/>
-      <c r="Y46" s="1" t="n"/>
-      <c r="Z46" s="1" t="n"/>
-      <c r="AA46" s="1" t="n"/>
-      <c r="AB46" s="1" t="n"/>
-      <c r="AC46" s="1" t="n"/>
-      <c r="AD46" s="1" t="n"/>
-      <c r="AE46" s="1" t="n"/>
-      <c r="AF46" s="1" t="n"/>
-      <c r="AG46" s="1" t="n"/>
-      <c r="AH46" s="1" t="n"/>
-      <c r="AI46" s="1" t="n"/>
+      <c r="B46" s="116" t="n"/>
+      <c r="C46" s="116" t="n"/>
+      <c r="D46" s="120" t="n"/>
+      <c r="E46" s="109">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,1),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="109">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,2),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="109">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,3),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="H46" s="109">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,4),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="I46" s="109">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,5),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="J46" s="109">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,6),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="109">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,7),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="109">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,8),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="109">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,9),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="N46" s="109">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,10),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="O46" s="109">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,11),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="P46" s="109">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,12),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Q46" s="109">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,13),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="R46" s="109">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,14),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="S46" s="109">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,15),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="T46" s="109">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,16),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="U46" s="109">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,17),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="V46" s="109">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,18),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="W46" s="109">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,19),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="X46" s="109">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,20),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Y46" s="109">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,21),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="Z46" s="109">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,22),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AA46" s="109">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,23),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AB46" s="109">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,24),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AC46" s="109">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,25),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AD46" s="109">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,26),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AE46" s="109">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,27),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AF46" s="109">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,28),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AG46" s="109">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,29),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AH46" s="109">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,30),"ddd"),"")</f>
+        <v/>
+      </c>
+      <c r="AI46" s="109">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,31),"ddd"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A47" s="115" t="n"/>
-      <c r="B47" s="116" t="n"/>
-      <c r="C47" s="116" t="n"/>
-      <c r="D47" s="119" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="3" t="n"/>
-      <c r="J47" s="4" t="n"/>
-      <c r="K47" s="4" t="n"/>
-      <c r="L47" s="3" t="n"/>
-      <c r="M47" s="4" t="n"/>
-      <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="n"/>
-      <c r="P47" s="2" t="n"/>
-      <c r="Q47" s="2" t="n"/>
-      <c r="R47" s="2" t="n"/>
-      <c r="S47" s="2" t="n"/>
-      <c r="T47" s="2" t="n"/>
-      <c r="U47" s="2" t="n"/>
-      <c r="V47" s="2" t="n"/>
-      <c r="W47" s="2" t="n"/>
-      <c r="X47" s="2" t="n"/>
-      <c r="Y47" s="2" t="n"/>
-      <c r="Z47" s="2" t="n"/>
-      <c r="AA47" s="2" t="n"/>
-      <c r="AB47" s="2" t="n"/>
-      <c r="AC47" s="2" t="n"/>
-      <c r="AD47" s="2" t="n"/>
-      <c r="AE47" s="2" t="n"/>
-      <c r="AF47" s="2" t="n"/>
-      <c r="AG47" s="2" t="n"/>
-      <c r="AH47" s="2" t="n"/>
-      <c r="AI47" s="2" t="n"/>
+      <c r="A47" s="117" t="n"/>
+      <c r="B47" s="118" t="n"/>
+      <c r="C47" s="118" t="n"/>
+      <c r="D47" s="121" t="n"/>
+      <c r="E47" s="112">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),1,"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="112">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),2,"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="112">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),3,"")</f>
+        <v/>
+      </c>
+      <c r="H47" s="112">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),4,"")</f>
+        <v/>
+      </c>
+      <c r="I47" s="112">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),5,"")</f>
+        <v/>
+      </c>
+      <c r="J47" s="112">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),6,"")</f>
+        <v/>
+      </c>
+      <c r="K47" s="112">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),7,"")</f>
+        <v/>
+      </c>
+      <c r="L47" s="112">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),8,"")</f>
+        <v/>
+      </c>
+      <c r="M47" s="112">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),9,"")</f>
+        <v/>
+      </c>
+      <c r="N47" s="112">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),10,"")</f>
+        <v/>
+      </c>
+      <c r="O47" s="112">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),11,"")</f>
+        <v/>
+      </c>
+      <c r="P47" s="112">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),12,"")</f>
+        <v/>
+      </c>
+      <c r="Q47" s="112">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),13,"")</f>
+        <v/>
+      </c>
+      <c r="R47" s="112">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),14,"")</f>
+        <v/>
+      </c>
+      <c r="S47" s="112">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),15,"")</f>
+        <v/>
+      </c>
+      <c r="T47" s="112">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),16,"")</f>
+        <v/>
+      </c>
+      <c r="U47" s="112">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),17,"")</f>
+        <v/>
+      </c>
+      <c r="V47" s="112">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),18,"")</f>
+        <v/>
+      </c>
+      <c r="W47" s="112">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),19,"")</f>
+        <v/>
+      </c>
+      <c r="X47" s="112">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),20,"")</f>
+        <v/>
+      </c>
+      <c r="Y47" s="112">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),21,"")</f>
+        <v/>
+      </c>
+      <c r="Z47" s="112">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),22,"")</f>
+        <v/>
+      </c>
+      <c r="AA47" s="112">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),23,"")</f>
+        <v/>
+      </c>
+      <c r="AB47" s="112">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),24,"")</f>
+        <v/>
+      </c>
+      <c r="AC47" s="112">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),25,"")</f>
+        <v/>
+      </c>
+      <c r="AD47" s="112">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),26,"")</f>
+        <v/>
+      </c>
+      <c r="AE47" s="112">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),27,"")</f>
+        <v/>
+      </c>
+      <c r="AF47" s="112">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),28,"")</f>
+        <v/>
+      </c>
+      <c r="AG47" s="112">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),29,"")</f>
+        <v/>
+      </c>
+      <c r="AH47" s="112">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),30,"")</f>
+        <v/>
+      </c>
+      <c r="AI47" s="112">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),31,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="16.2" customHeight="1" thickBot="1">
       <c r="A48" s="9" t="n">
@@ -4165,9 +4899,9 @@
       <c r="C59" s="37" t="n"/>
       <c r="D59" s="40" t="n"/>
       <c r="E59" s="6" t="n"/>
-      <c r="F59" s="121" t="n"/>
-      <c r="G59" s="121" t="n"/>
-      <c r="H59" s="122" t="n"/>
+      <c r="F59" s="123" t="n"/>
+      <c r="G59" s="123" t="n"/>
+      <c r="H59" s="124" t="n"/>
       <c r="I59" s="23" t="n"/>
       <c r="J59" s="6" t="n"/>
       <c r="K59" s="6" t="n"/>
@@ -4204,9 +4938,9 @@
       <c r="C60" s="37" t="n"/>
       <c r="D60" s="40" t="n"/>
       <c r="E60" s="6" t="n"/>
-      <c r="F60" s="121" t="n"/>
-      <c r="G60" s="121" t="n"/>
-      <c r="H60" s="122" t="n"/>
+      <c r="F60" s="123" t="n"/>
+      <c r="G60" s="123" t="n"/>
+      <c r="H60" s="124" t="n"/>
       <c r="I60" s="23" t="n"/>
       <c r="J60" s="6" t="n"/>
       <c r="K60" s="6" t="n"/>
@@ -4279,9 +5013,9 @@
       <c r="C62" s="37" t="n"/>
       <c r="D62" s="40" t="n"/>
       <c r="E62" s="6" t="n"/>
-      <c r="F62" s="121" t="n"/>
-      <c r="G62" s="121" t="n"/>
-      <c r="H62" s="122" t="n"/>
+      <c r="F62" s="123" t="n"/>
+      <c r="G62" s="123" t="n"/>
+      <c r="H62" s="124" t="n"/>
       <c r="I62" s="23" t="n"/>
       <c r="J62" s="6" t="n"/>
       <c r="K62" s="6" t="n"/>
@@ -4318,9 +5052,9 @@
       <c r="C63" s="37" t="n"/>
       <c r="D63" s="40" t="n"/>
       <c r="E63" s="6" t="n"/>
-      <c r="F63" s="121" t="n"/>
-      <c r="G63" s="121" t="n"/>
-      <c r="H63" s="122" t="n"/>
+      <c r="F63" s="123" t="n"/>
+      <c r="G63" s="123" t="n"/>
+      <c r="H63" s="124" t="n"/>
       <c r="I63" s="23" t="n"/>
       <c r="J63" s="6" t="n"/>
       <c r="K63" s="6" t="n"/>
@@ -4357,9 +5091,9 @@
       <c r="C64" s="37" t="n"/>
       <c r="D64" s="40" t="n"/>
       <c r="E64" s="6" t="n"/>
-      <c r="F64" s="121" t="n"/>
-      <c r="G64" s="121" t="n"/>
-      <c r="H64" s="122" t="n"/>
+      <c r="F64" s="123" t="n"/>
+      <c r="G64" s="123" t="n"/>
+      <c r="H64" s="124" t="n"/>
       <c r="I64" s="23" t="n"/>
       <c r="J64" s="6" t="n"/>
       <c r="K64" s="6" t="n"/>
@@ -4396,9 +5130,9 @@
       <c r="C65" s="37" t="n"/>
       <c r="D65" s="40" t="n"/>
       <c r="E65" s="6" t="n"/>
-      <c r="F65" s="121" t="n"/>
-      <c r="G65" s="121" t="n"/>
-      <c r="H65" s="122" t="n"/>
+      <c r="F65" s="123" t="n"/>
+      <c r="G65" s="123" t="n"/>
+      <c r="H65" s="124" t="n"/>
       <c r="I65" s="23" t="n"/>
       <c r="J65" s="6" t="n"/>
       <c r="K65" s="6" t="n"/>
@@ -4434,7 +5168,7 @@
       <c r="B66" s="37" t="n"/>
       <c r="C66" s="37" t="n"/>
       <c r="D66" s="40" t="n"/>
-      <c r="E66" s="137" t="n"/>
+      <c r="E66" s="148" t="n"/>
       <c r="F66" s="7" t="n"/>
       <c r="G66" s="7" t="n"/>
       <c r="H66" s="23" t="n"/>
@@ -4473,7 +5207,7 @@
       <c r="B67" s="37" t="n"/>
       <c r="C67" s="37" t="n"/>
       <c r="D67" s="40" t="n"/>
-      <c r="E67" s="137" t="n"/>
+      <c r="E67" s="148" t="n"/>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="n"/>
       <c r="H67" s="23" t="n"/>
@@ -4512,7 +5246,7 @@
       <c r="B68" s="37" t="n"/>
       <c r="C68" s="37" t="n"/>
       <c r="D68" s="40" t="n"/>
-      <c r="E68" s="137" t="n"/>
+      <c r="E68" s="148" t="n"/>
       <c r="F68" s="7" t="n"/>
       <c r="G68" s="7" t="n"/>
       <c r="H68" s="23" t="n"/>
@@ -4551,7 +5285,7 @@
       <c r="B69" s="37" t="n"/>
       <c r="C69" s="37" t="n"/>
       <c r="D69" s="40" t="n"/>
-      <c r="E69" s="137" t="n"/>
+      <c r="E69" s="148" t="n"/>
       <c r="F69" s="7" t="n"/>
       <c r="G69" s="7" t="n"/>
       <c r="H69" s="23" t="n"/>
@@ -4590,7 +5324,7 @@
       <c r="B70" s="37" t="n"/>
       <c r="C70" s="37" t="n"/>
       <c r="D70" s="40" t="n"/>
-      <c r="E70" s="137" t="n"/>
+      <c r="E70" s="148" t="n"/>
       <c r="F70" s="7" t="n"/>
       <c r="G70" s="7" t="n"/>
       <c r="H70" s="23" t="n"/>
@@ -4629,7 +5363,7 @@
       <c r="B71" s="37" t="n"/>
       <c r="C71" s="37" t="n"/>
       <c r="D71" s="40" t="n"/>
-      <c r="E71" s="137" t="n"/>
+      <c r="E71" s="148" t="n"/>
       <c r="F71" s="7" t="n"/>
       <c r="G71" s="7" t="n"/>
       <c r="H71" s="23" t="n"/>
@@ -4715,275 +5449,275 @@
       <c r="O73" s="14" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" thickBot="1">
-      <c r="A74" s="123" t="inlineStr">
+      <c r="A74" s="125" t="inlineStr">
         <is>
           <t>TOTAL DAILY CREWS MANPOWER</t>
         </is>
       </c>
-      <c r="B74" s="114" t="n"/>
-      <c r="C74" s="118" t="n"/>
-      <c r="D74" s="117" t="inlineStr">
+      <c r="B74" s="116" t="n"/>
+      <c r="C74" s="120" t="n"/>
+      <c r="D74" s="119" t="inlineStr">
         <is>
           <t>SHIFT</t>
         </is>
       </c>
-      <c r="E74" s="1">
+      <c r="E74" s="109">
         <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,1),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="F74" s="1">
+      <c r="F74" s="109">
         <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,2),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="G74" s="1">
+      <c r="G74" s="109">
         <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,3),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="H74" s="1">
+      <c r="H74" s="109">
         <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,4),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="I74" s="1">
+      <c r="I74" s="109">
         <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,5),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="109">
         <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,6),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="109">
         <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,7),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="L74" s="1">
+      <c r="L74" s="109">
         <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,8),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="M74" s="1">
+      <c r="M74" s="109">
         <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,9),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="N74" s="1">
+      <c r="N74" s="109">
         <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,10),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="O74" s="1">
+      <c r="O74" s="109">
         <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,11),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="109">
         <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,12),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Q74" s="1">
+      <c r="Q74" s="109">
         <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,13),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="R74" s="1">
+      <c r="R74" s="109">
         <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,14),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="S74" s="1">
+      <c r="S74" s="109">
         <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,15),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="T74" s="1">
+      <c r="T74" s="109">
         <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,16),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="U74" s="1">
+      <c r="U74" s="109">
         <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,17),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="V74" s="1">
+      <c r="V74" s="109">
         <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,18),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="W74" s="1">
+      <c r="W74" s="109">
         <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,19),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="X74" s="1">
+      <c r="X74" s="109">
         <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,20),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Y74" s="1">
+      <c r="Y74" s="109">
         <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,21),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Z74" s="1">
+      <c r="Z74" s="109">
         <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,22),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AA74" s="1">
+      <c r="AA74" s="109">
         <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,23),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AB74" s="1">
+      <c r="AB74" s="109">
         <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,24),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AC74" s="1">
+      <c r="AC74" s="109">
         <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,25),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AD74" s="1">
+      <c r="AD74" s="109">
         <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,26),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AE74" s="1">
+      <c r="AE74" s="109">
         <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,27),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AF74" s="1">
+      <c r="AF74" s="109">
         <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,28),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AG74" s="1">
+      <c r="AG74" s="109">
         <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,29),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AH74" s="1">
+      <c r="AH74" s="109">
         <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,30),"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AI74" s="1">
+      <c r="AI74" s="109">
         <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),TEXT(DATE($AL$5,$AP$2,31),"ddd"),"")</f>
         <v/>
       </c>
     </row>
     <row r="75" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A75" s="110" t="n"/>
-      <c r="C75" s="124" t="n"/>
+      <c r="A75" s="111" t="n"/>
+      <c r="C75" s="126" t="n"/>
       <c r="D75" s="105" t="n"/>
-      <c r="E75" s="2">
+      <c r="E75" s="112">
         <f>IF(1&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),1,"")</f>
         <v/>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="112">
         <f>IF(2&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),2,"")</f>
         <v/>
       </c>
-      <c r="G75" s="2">
+      <c r="G75" s="112">
         <f>IF(3&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),3,"")</f>
         <v/>
       </c>
-      <c r="H75" s="2">
+      <c r="H75" s="112">
         <f>IF(4&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),4,"")</f>
         <v/>
       </c>
-      <c r="I75" s="3">
+      <c r="I75" s="112">
         <f>IF(5&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),5,"")</f>
         <v/>
       </c>
-      <c r="J75" s="4">
+      <c r="J75" s="112">
         <f>IF(6&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),6,"")</f>
         <v/>
       </c>
-      <c r="K75" s="4">
+      <c r="K75" s="112">
         <f>IF(7&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),7,"")</f>
         <v/>
       </c>
-      <c r="L75" s="3">
+      <c r="L75" s="112">
         <f>IF(8&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),8,"")</f>
         <v/>
       </c>
-      <c r="M75" s="4">
+      <c r="M75" s="112">
         <f>IF(9&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),9,"")</f>
         <v/>
       </c>
-      <c r="N75" s="2">
+      <c r="N75" s="112">
         <f>IF(10&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),10,"")</f>
         <v/>
       </c>
-      <c r="O75" s="2">
+      <c r="O75" s="112">
         <f>IF(11&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),11,"")</f>
         <v/>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="112">
         <f>IF(12&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),12,"")</f>
         <v/>
       </c>
-      <c r="Q75" s="2">
+      <c r="Q75" s="112">
         <f>IF(13&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),13,"")</f>
         <v/>
       </c>
-      <c r="R75" s="2">
+      <c r="R75" s="112">
         <f>IF(14&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),14,"")</f>
         <v/>
       </c>
-      <c r="S75" s="2">
+      <c r="S75" s="112">
         <f>IF(15&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),15,"")</f>
         <v/>
       </c>
-      <c r="T75" s="2">
+      <c r="T75" s="112">
         <f>IF(16&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),16,"")</f>
         <v/>
       </c>
-      <c r="U75" s="2">
+      <c r="U75" s="112">
         <f>IF(17&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),17,"")</f>
         <v/>
       </c>
-      <c r="V75" s="2">
+      <c r="V75" s="112">
         <f>IF(18&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),18,"")</f>
         <v/>
       </c>
-      <c r="W75" s="2">
+      <c r="W75" s="112">
         <f>IF(19&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),19,"")</f>
         <v/>
       </c>
-      <c r="X75" s="2">
+      <c r="X75" s="112">
         <f>IF(20&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),20,"")</f>
         <v/>
       </c>
-      <c r="Y75" s="2">
+      <c r="Y75" s="112">
         <f>IF(21&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),21,"")</f>
         <v/>
       </c>
-      <c r="Z75" s="2">
+      <c r="Z75" s="112">
         <f>IF(22&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),22,"")</f>
         <v/>
       </c>
-      <c r="AA75" s="2">
+      <c r="AA75" s="112">
         <f>IF(23&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),23,"")</f>
         <v/>
       </c>
-      <c r="AB75" s="2">
+      <c r="AB75" s="112">
         <f>IF(24&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),24,"")</f>
         <v/>
       </c>
-      <c r="AC75" s="2">
+      <c r="AC75" s="112">
         <f>IF(25&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),25,"")</f>
         <v/>
       </c>
-      <c r="AD75" s="2">
+      <c r="AD75" s="112">
         <f>IF(26&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),26,"")</f>
         <v/>
       </c>
-      <c r="AE75" s="2">
+      <c r="AE75" s="112">
         <f>IF(27&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),27,"")</f>
         <v/>
       </c>
-      <c r="AF75" s="2">
+      <c r="AF75" s="112">
         <f>IF(28&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),28,"")</f>
         <v/>
       </c>
-      <c r="AG75" s="2">
+      <c r="AG75" s="112">
         <f>IF(29&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),29,"")</f>
         <v/>
       </c>
-      <c r="AH75" s="2">
+      <c r="AH75" s="112">
         <f>IF(30&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),30,"")</f>
         <v/>
       </c>
-      <c r="AI75" s="2">
+      <c r="AI75" s="112">
         <f>IF(31&lt;=DAY(EOMONTH(DATE($AL$5,$AP$2,1),0)),31,"")</f>
         <v/>
       </c>
     </row>
     <row r="76" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A76" s="110" t="n"/>
-      <c r="C76" s="124" t="n"/>
+      <c r="A76" s="111" t="n"/>
+      <c r="C76" s="126" t="n"/>
       <c r="D76" s="15" t="inlineStr">
         <is>
           <t>D</t>
@@ -5115,8 +5849,8 @@
       </c>
     </row>
     <row r="77" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A77" s="110" t="n"/>
-      <c r="C77" s="124" t="n"/>
+      <c r="A77" s="111" t="n"/>
+      <c r="C77" s="126" t="n"/>
       <c r="D77" s="17" t="inlineStr">
         <is>
           <t>T</t>
@@ -5248,9 +5982,9 @@
       </c>
     </row>
     <row r="78" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A78" s="115" t="n"/>
-      <c r="B78" s="116" t="n"/>
-      <c r="C78" s="119" t="n"/>
+      <c r="A78" s="117" t="n"/>
+      <c r="B78" s="118" t="n"/>
+      <c r="C78" s="121" t="n"/>
       <c r="D78" s="19" t="inlineStr">
         <is>
           <t>G</t>
@@ -5383,7 +6117,7 @@
     </row>
     <row r="79" ht="15" customHeight="1" thickBot="1"/>
     <row r="80" ht="21" customHeight="1" thickBot="1">
-      <c r="E80" s="117" t="inlineStr">
+      <c r="E80" s="119" t="inlineStr">
         <is>
           <t>SHIFT</t>
         </is>
@@ -5395,7 +6129,7 @@
       <c r="J80" s="104" t="n"/>
     </row>
     <row r="81" ht="16.2" customHeight="1" thickBot="1">
-      <c r="E81" s="44" t="inlineStr">
+      <c r="E81" s="127" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -5411,7 +6145,7 @@
       <c r="J81" s="104" t="n"/>
     </row>
     <row r="82" ht="16.2" customHeight="1" thickBot="1">
-      <c r="E82" s="45" t="inlineStr">
+      <c r="E82" s="128" t="inlineStr">
         <is>
           <t>T</t>
         </is>
@@ -5430,30 +6164,34 @@
           <t>ABDULLAH A. ALSHEHRY</t>
         </is>
       </c>
-      <c r="N82" s="116" t="n"/>
-      <c r="O82" s="116" t="n"/>
-      <c r="P82" s="116" t="n"/>
-      <c r="Q82" s="116" t="n"/>
-      <c r="R82" s="116" t="n"/>
-      <c r="S82" s="116" t="n"/>
+      <c r="N82" s="118" t="n"/>
+      <c r="O82" s="118" t="n"/>
+      <c r="P82" s="118" t="n"/>
+      <c r="Q82" s="118" t="n"/>
+      <c r="R82" s="118" t="n"/>
+      <c r="S82" s="118" t="n"/>
       <c r="W82" s="96">
         <f>UPPER(TEXT(TODAY(),"DDDD dd/mm/yyyy"))</f>
         <v/>
       </c>
-      <c r="X82" s="116" t="n"/>
-      <c r="Y82" s="116" t="n"/>
-      <c r="Z82" s="116" t="n"/>
-      <c r="AA82" s="116" t="n"/>
-      <c r="AB82" s="116" t="n"/>
-      <c r="AC82" s="116" t="n"/>
+      <c r="X82" s="118" t="n"/>
+      <c r="Y82" s="118" t="n"/>
+      <c r="Z82" s="118" t="n"/>
+      <c r="AA82" s="118" t="n"/>
+      <c r="AB82" s="118" t="n"/>
+      <c r="AC82" s="118" t="n"/>
     </row>
     <row r="83" ht="16.2" customHeight="1" thickBot="1">
-      <c r="E83" s="46" t="inlineStr">
+      <c r="E83" s="129" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F83" s="20" t="n"/>
+      <c r="F83" s="20" t="inlineStr">
+        <is>
+          <t>GRV (23:00 - 07:00)</t>
+        </is>
+      </c>
       <c r="G83" s="103" t="n"/>
       <c r="H83" s="103" t="n"/>
       <c r="I83" s="103" t="n"/>
@@ -5470,120 +6208,184 @@
       </c>
     </row>
     <row r="85">
-      <c r="E85" s="125" t="inlineStr">
+      <c r="E85" s="130" t="inlineStr">
         <is>
-          <t>ADDITIONAL CODES</t>
+          <t>CODE LEGEND — ALL CODES</t>
         </is>
       </c>
     </row>
     <row r="86" ht="16" customHeight="1">
-      <c r="E86" s="126" t="inlineStr">
+      <c r="E86" s="131" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F86" s="132" t="inlineStr">
+        <is>
+          <t>DAY</t>
+        </is>
+      </c>
+      <c r="K86" s="133" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="L86" s="132" t="inlineStr">
+        <is>
+          <t>TWILIGHT</t>
+        </is>
+      </c>
+      <c r="Q86" s="134" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="R86" s="132" t="inlineStr">
+        <is>
+          <t>GRAVEYARD</t>
+        </is>
+      </c>
+      <c r="W86" s="135" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="X86" s="132" t="inlineStr">
+        <is>
+          <t>TRAINING</t>
+        </is>
+      </c>
+      <c r="AC86" s="136" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="AD86" s="132" t="inlineStr">
+        <is>
+          <t>VACATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="16" customHeight="1">
+      <c r="E87" s="137" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F87" s="132" t="inlineStr">
+        <is>
+          <t>REST/RDO</t>
+        </is>
+      </c>
+      <c r="K87" s="138" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F86" s="127" t="inlineStr">
+      <c r="L87" s="132" t="inlineStr">
         <is>
           <t>ABSENT</t>
         </is>
       </c>
-      <c r="L86" s="128" t="inlineStr">
+      <c r="Q87" s="139" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="M86" s="127" t="inlineStr">
+      <c r="R87" s="132" t="inlineStr">
         <is>
           <t>HOLIDAY</t>
         </is>
       </c>
-      <c r="S86" s="129" t="inlineStr">
+      <c r="W87" s="140" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="T86" s="127" t="inlineStr">
+      <c r="X87" s="132" t="inlineStr">
         <is>
           <t>OVERTIME</t>
         </is>
       </c>
-      <c r="Z86" s="130" t="inlineStr">
+      <c r="AC87" s="141" t="inlineStr">
         <is>
           <t>OS</t>
         </is>
       </c>
-      <c r="AA86" s="127" t="inlineStr">
+      <c r="AD87" s="132" t="inlineStr">
         <is>
           <t>OUTSTATION</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="16" customHeight="1">
-      <c r="E87" s="131" t="inlineStr">
+    <row r="88" ht="16" customHeight="1">
+      <c r="E88" s="142" t="inlineStr">
         <is>
           <t>S/L</t>
         </is>
       </c>
-      <c r="F87" s="127" t="inlineStr">
+      <c r="F88" s="132" t="inlineStr">
         <is>
           <t>SICK LEAVE</t>
         </is>
       </c>
-      <c r="L87" s="132" t="inlineStr">
+      <c r="K88" s="143" t="inlineStr">
         <is>
           <t>C/T</t>
         </is>
       </c>
-      <c r="M87" s="127" t="inlineStr">
+      <c r="L88" s="132" t="inlineStr">
         <is>
           <t>COMP TIME</t>
         </is>
       </c>
-      <c r="S87" s="133" t="inlineStr">
+      <c r="Q88" s="144" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="T87" s="127" t="inlineStr">
+      <c r="R88" s="132" t="inlineStr">
         <is>
           <t>LATE/LEAVE</t>
         </is>
       </c>
-      <c r="Z87" s="134" t="inlineStr">
+      <c r="W88" s="145" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="AA87" s="127" t="inlineStr">
+      <c r="X88" s="132" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="39">
-    <mergeCell ref="M87:Q87"/>
-    <mergeCell ref="F87:J87"/>
+  <mergeCells count="45">
+    <mergeCell ref="X88:AA88"/>
     <mergeCell ref="E2:AC2"/>
     <mergeCell ref="C1:C2"/>
+    <mergeCell ref="AD87:AG87"/>
     <mergeCell ref="AK6:AN6"/>
     <mergeCell ref="A74:C78"/>
     <mergeCell ref="W82:AC82"/>
-    <mergeCell ref="AA87:AE87"/>
     <mergeCell ref="E80:J80"/>
     <mergeCell ref="F83:J83"/>
-    <mergeCell ref="AA86:AE86"/>
-    <mergeCell ref="T87:X87"/>
+    <mergeCell ref="F88:I88"/>
+    <mergeCell ref="L86:O86"/>
     <mergeCell ref="AL5:AN5"/>
     <mergeCell ref="A46:D47"/>
     <mergeCell ref="AD1:AI2"/>
     <mergeCell ref="A3:D4"/>
-    <mergeCell ref="F86:J86"/>
+    <mergeCell ref="F87:I87"/>
     <mergeCell ref="E62:H62"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="M83:S83"/>
+    <mergeCell ref="X86:AA86"/>
     <mergeCell ref="AL4:AN4"/>
+    <mergeCell ref="R88:U88"/>
     <mergeCell ref="E64:H64"/>
+    <mergeCell ref="R87:U87"/>
     <mergeCell ref="F81:J81"/>
     <mergeCell ref="A22:D23"/>
     <mergeCell ref="D74:D75"/>
@@ -5591,103 +6393,68 @@
     <mergeCell ref="A42:D43"/>
     <mergeCell ref="AK3:AN3"/>
     <mergeCell ref="M82:S82"/>
-    <mergeCell ref="M86:Q86"/>
+    <mergeCell ref="L87:O87"/>
+    <mergeCell ref="X87:AA87"/>
+    <mergeCell ref="F86:I86"/>
     <mergeCell ref="E63:H63"/>
     <mergeCell ref="E60:H60"/>
     <mergeCell ref="E1:AC1"/>
     <mergeCell ref="E65:H65"/>
-    <mergeCell ref="T86:X86"/>
+    <mergeCell ref="L88:O88"/>
     <mergeCell ref="F82:J82"/>
+    <mergeCell ref="R86:U86"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E59:H59"/>
+    <mergeCell ref="AD86:AG86"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E21:O21 E24:AI40 E44:AI44 E45:O45 E48:AI56 E57:E72 E73:O73 I57:AI72">
-    <cfRule type="containsText" priority="13" operator="containsText" dxfId="5" text="TR">
-      <formula>NOT(ISERROR(SEARCH("TR",E21)))</formula>
+  <conditionalFormatting sqref="E5:AI73">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
+      <formula>"D"</formula>
     </cfRule>
-    <cfRule type="containsText" priority="14" operator="containsText" dxfId="4" text="V">
-      <formula>NOT(ISERROR(SEARCH("V",E21)))</formula>
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
+      <formula>"T"</formula>
     </cfRule>
-    <cfRule type="containsText" priority="15" operator="containsText" dxfId="3" text="R">
-      <formula>NOT(ISERROR(SEARCH("R",E21)))</formula>
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
+      <formula>"G"</formula>
     </cfRule>
-    <cfRule type="containsText" priority="16" operator="containsText" dxfId="2" text="G">
-      <formula>NOT(ISERROR(SEARCH("G",E21)))</formula>
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="15">
+      <formula>"TR"</formula>
     </cfRule>
-    <cfRule type="containsText" priority="17" operator="containsText" dxfId="1" text="T">
-      <formula>NOT(ISERROR(SEARCH("T",E21)))</formula>
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="16">
+      <formula>"V"</formula>
     </cfRule>
-    <cfRule type="containsText" priority="18" operator="containsText" dxfId="0" text="D">
-      <formula>NOT(ISERROR(SEARCH("D",E21)))</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="17">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="18">
       <formula>"H"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="19">
       <formula>"OT"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="16" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="21" operator="equal" dxfId="20">
       <formula>"OS"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="16">
+    <cfRule type="cellIs" priority="22" operator="equal" dxfId="21">
       <formula>"S/L"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="17">
+    <cfRule type="cellIs" priority="23" operator="equal" dxfId="22">
       <formula>"C/T"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="18">
+    <cfRule type="cellIs" priority="24" operator="equal" dxfId="23">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="19">
+    <cfRule type="cellIs" priority="25" operator="equal" dxfId="24">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:AI20">
-    <cfRule type="containsText" priority="1" operator="containsText" dxfId="5" text="TR">
-      <formula>NOT(ISERROR(SEARCH("TR",E5)))</formula>
+  <conditionalFormatting sqref="A5:D73">
+    <cfRule type="expression" priority="26" dxfId="25">
+      <formula>$D5="OJT"</formula>
     </cfRule>
-    <cfRule type="containsText" priority="2" operator="containsText" dxfId="4" text="V">
-      <formula>NOT(ISERROR(SEARCH("V",E5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" dxfId="3" text="R">
-      <formula>NOT(ISERROR(SEARCH("R",E5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" priority="4" operator="containsText" dxfId="2" text="G">
-      <formula>NOT(ISERROR(SEARCH("G",E5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" priority="5" operator="containsText" dxfId="1" text="T">
-      <formula>NOT(ISERROR(SEARCH("T",E5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" priority="6" operator="containsText" dxfId="0" text="D">
-      <formula>NOT(ISERROR(SEARCH("D",E5)))</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="21" operator="equal" dxfId="12">
-      <formula>"A"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="22" operator="equal" dxfId="13">
-      <formula>"H"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="23" operator="equal" dxfId="14">
-      <formula>"OT"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="24" operator="equal" dxfId="15">
-      <formula>"OS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="25" operator="equal" dxfId="16">
-      <formula>"S/L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="26" operator="equal" dxfId="17">
-      <formula>"C/T"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="27" operator="equal" dxfId="18">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="28" operator="equal" dxfId="19">
-      <formula>"N"</formula>
+    <cfRule type="expression" priority="27" dxfId="26">
+      <formula>$D5="ACT/SUPV"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>

</xml_diff>